<commit_message>
fix(upload): y-axis padding + UX prose + REST demo row (#69 #70 #71)
#69 - Add layout.padding.left=90 + ticks.autoSkip=false + ticks.padding=8
       so all 23 district y-axis labels are visible.
       Also set maintainAspectRatio:false to honour canvas height from #66.
#70 - Replace user-facing 'Fix A + Fix B' jargon with 'static-lookup steps'
       (EN) and 'statischen Suchschritten' (DE). Also updated fuzzy error
       banner innerHTML and setProgress() message. Code comments retain
       'Fix A:'-style internal markers.
#71 - Add row 13 to sample_acd_test.xlsx with abbreviated street name
       'Klosterneub. Str.' (PLZ 1070) that exercises the REST-API fallback
       path, so demo users can verify match_quality = rest_api_fallback.
       Banner updated to '13-row sample' with REST demo hint text.

Closes #69 #70 #71.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data/sample_acd_test.xlsx
+++ b/docs/data/sample_acd_test.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabelle2" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,41 +425,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ObjektNr.</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>PLZ</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Strasse</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>HausNr</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Stiege/RH</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ACD Code</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>_demo_note</t>
         </is>
@@ -471,6 +483,7 @@
       <c r="E2" t="n">
         <v>1</v>
       </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>match — Bezirk 21</t>
@@ -497,6 +510,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>match — Bezirk 21</t>
@@ -523,6 +537,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>match — Bezirk 21</t>
@@ -549,6 +564,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>match — Bezirk 22</t>
@@ -575,6 +591,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>match — Bezirk 22</t>
@@ -601,6 +618,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>focus — Bezirk 20</t>
@@ -627,6 +645,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>focus — Bezirk 20</t>
@@ -653,6 +672,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>central — Bezirk 01</t>
@@ -679,6 +699,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>central — Bezirk 01</t>
@@ -707,6 +728,7 @@
           <t>Weg 1</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>garden plot — composite address</t>
@@ -733,6 +755,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>deliberate miss — street not in city</t>
@@ -759,9 +782,35 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>deliberate miss — house number unrealistic</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>1070</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Klosterneub. Str.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>REST demo — abbreviated street triggers rest_api_fallback</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(upload): y-axis padding + UX prose + REST demo row (#69 #70 #71) (#72)
#69 - Add layout.padding.left=90 + ticks.autoSkip=false + ticks.padding=8
       so all 23 district y-axis labels are visible.
       Also set maintainAspectRatio:false to honour canvas height from #66.
#70 - Replace user-facing 'Fix A + Fix B' jargon with 'static-lookup steps'
       (EN) and 'statischen Suchschritten' (DE). Also updated fuzzy error
       banner innerHTML and setProgress() message. Code comments retain
       'Fix A:'-style internal markers.
#71 - Add row 13 to sample_acd_test.xlsx with abbreviated street name
       'Klosterneub. Str.' (PLZ 1070) that exercises the REST-API fallback
       path, so demo users can verify match_quality = rest_api_fallback.
       Banner updated to '13-row sample' with REST demo hint text.

Closes #69 #70 #71.

Co-authored-by: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data/sample_acd_test.xlsx
+++ b/docs/data/sample_acd_test.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabelle2" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,41 +425,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ObjektNr.</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>PLZ</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Strasse</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>HausNr</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Stiege/RH</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ACD Code</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>_demo_note</t>
         </is>
@@ -471,6 +483,7 @@
       <c r="E2" t="n">
         <v>1</v>
       </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>match — Bezirk 21</t>
@@ -497,6 +510,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>match — Bezirk 21</t>
@@ -523,6 +537,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>match — Bezirk 21</t>
@@ -549,6 +564,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>match — Bezirk 22</t>
@@ -575,6 +591,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>match — Bezirk 22</t>
@@ -601,6 +618,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>focus — Bezirk 20</t>
@@ -627,6 +645,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>focus — Bezirk 20</t>
@@ -653,6 +672,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>central — Bezirk 01</t>
@@ -679,6 +699,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>central — Bezirk 01</t>
@@ -707,6 +728,7 @@
           <t>Weg 1</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>garden plot — composite address</t>
@@ -733,6 +755,7 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>deliberate miss — street not in city</t>
@@ -759,9 +782,35 @@
           <t xml:space="preserve">  </t>
         </is>
       </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>deliberate miss — house number unrealistic</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>1070</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Klosterneub. Str.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>REST demo — abbreviated street triggers rest_api_fallback</t>
         </is>
       </c>
     </row>

</xml_diff>